<commit_message>
Revert "Keep the LOCAL median where a case holds both (issue #21 sec 5.1)"
This reverts commit 2e8f5efa66ac174539d63f98b9674e10d444bde1.
</commit_message>
<xml_diff>
--- a/outputs/master_rename_build/tables/nsu_reference_set.xlsx
+++ b/outputs/master_rename_build/tables/nsu_reference_set.xlsx
@@ -104933,10 +104933,10 @@
         <v>191</v>
       </c>
       <c r="G2543" s="1">
-        <v>325</v>
+        <v>425</v>
       </c>
       <c r="H2543" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2543" t="s">
         <v>200</v>
@@ -105056,10 +105056,10 @@
         <v>191</v>
       </c>
       <c r="G2546" s="1">
-        <v>150</v>
+        <v>137.5</v>
       </c>
       <c r="H2546" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2546" t="s">
         <v>200</v>

</xml_diff>